<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-05 La chaussette de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-05.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>escalier de bois, classe, radiateur du soir</t>
+          <t>école puis maison, chaussette bleue sur la première marche, escalier de bois, lumière de cuisine, cacao</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, papa, maman, maîtresse</t>
+          <t>Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino trouve sa chaussette bleue, puis découpe une bande pareille à l'école. Un chuchotement serre son ventre. Le soir, il raconte près du cacao. Le lendemain, la chaussette l'attend, le ventre est calme.</t>
+          <t>Les casiers claquent. Sur la porte, un éclat de casier luit. Nino a un malaise, veut parler maintenant. Les mots se cognent à la classe. À la maison, la chaussette bleue tombe sur la première marche. Il parle trop vite près de la porte. Il refuse de foncer, raconte près de l'escalier. Merci vécu. Un éclat de casier reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une chaussette bleue attend sur la première marche. L'escalier en bois craque, tout doux. Une lumière ronde vient de la cuisine. Ça sent le cacao, un peu sucré. Maman chante tout bas, près de la casserole. Papa cherche l'autre chaussette sous le banc. La voilà. Elle s'était cachée. La bleue t'attendait, Nino. En ce moment, Nino s'assoit pour l'enfiler. La laine est un peu rêche, un peu chaude. Elle chatouille, papa. Tire jusqu'au talon. Et l'autre. Nino enfile la deuxième. Tes deux pieds sont au chaud. Merci, maman. À l'école, je veux découper une bande. Une bande bleue, comme la chaussette. Les ciseaux attendent dans la classe. Tu écoutes d'abord. Oui. Nino pose le pied sur la marche. L'escalier craque encore. À l'école, la classe sent les feuilles neuves. Bonjour. On range les ciseaux. Bonjour, maîtresse. Nino écoute. Il pose les ciseaux, les pointes en bas. Maintenant, on découpe une bande. Nino choisit le papier bleu. Il découpe tout doux. La bande tombe, longue et fine. Elle ressemble à ma chaussette. Oui, Nino. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Nino sent un malaise. Son ventre se serre. Il repose les mains sur ses genoux. Il reste près de sa chaise. La bande bleue attend sur la table. Le soir, la chaussette bleue sèche près du radiateur. La porte s'ouvre. Te voilà. Le cacao est prêt. Nino pose la bande bleue sur la marche. À côté de l'endroit de ce matin. Le ventre est encore serré.</t>
+          <t>Les casiers claquent dans le couloir. Le métal est froid, un peu lisse. Sur la porte, un éclat de casier luit. Il brille, papa. Tu le vois, sur le métal ? Nino accroche son manteau. Le crochet fait tic. Une étiquette pend au cartable. Elle est froide sous le doigt. Elle pique un peu. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Il part vers la porte. Une chaussette bleue dépasse du pantalon. La laine est un peu rêche. Elle chatouille. La classe sent les feuilles. Un banc de bois attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du banc. Il s'assoit, le dos droit. Un camarade s'approche du banc. Il parle tout près, d'un secret. Nino sent un malaise. Son ventre se serre, petit. Je n'aime pas ça. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. Le ventre reste serré. À la sortie, papa attend près des casiers. On rentre, Nino ? Oui. Nino touche l'éclat de casier, un instant. Le soir, la porte de la maison s'ouvre. Une lumière ronde vient de la cuisine. Ça sent le cacao, un peu sucré. L'escalier en bois craque. Nino retire la chaussette trop vite. Elle tombe sur la première marche. Te voilà, Nino. Le cacao est prêt. J'ai quelque chose, maintenant ! Nino avance trop vite vers la cuisine. Maman remue la casserole.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une chaussette bleue attend sur la première marche. L'escalier en bois craque, tout doux. Une lumière ronde vient de la cuisine. Ça sent le cacao, un peu sucré. Maman chante tout bas, près de la casserole. Papa cherche l'autre chaussette sous le banc. La voilà. Elle s'était cachée. La bleue t'attendait, Nino. En ce moment, Nino s'assoit pour l'enfiler. La laine est un peu rêche, un peu chaude. Elle chatouille, papa. Tire jusqu'au talon. Et l'autre. Nino enfile la deuxième. Tes deux pieds sont au chaud. Merci, maman. À l'école, je veux découper une bande. Une bande bleue, comme la chaussette. Les ciseaux attendent dans la classe. Tu écoutes d'abord. Oui. Nino pose le pied sur la marche. L'escalier craque encore. À l'école, la classe sent les feuilles neuves. Bonjour. On range les ciseaux. Bonjour, maîtresse. Nino écoute. Il pose les ciseaux, les pointes en bas. Maintenant, on découpe une bande. Nino choisit le papier bleu. Il découpe tout doux. La bande tombe, longue et fine. Elle ressemble à ma chaussette. Oui, Nino. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Nino sent un malaise. Son ventre se serre. Il repose les mains sur ses genoux. Il reste près de sa chaise. La bande bleue attend sur la table. Le soir, la chaussette bleue sèche près du radiateur. La porte s'ouvre. Te voilà. Le cacao est prêt. Nino pose la bande bleue sur la marche. À côté de l'endroit de ce matin. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les casiers claquent dans le couloir. Le métal est froid, un peu lisse. Sur la porte, un &lt;emphasis level="moderate"&gt;éclat de casier&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le métal ? Nino accroche son manteau. Le crochet fait tic. Une étiquette pend au cartable. Elle est froide sous le doigt. Elle pique un peu. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Il part vers la porte. Une chaussette bleue dépasse du pantalon. La laine est un peu rêche. Elle chatouille. La classe sent les feuilles. Un banc de bois attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du banc. Il s'assoit, le dos droit. Un camarade s'approche du banc. Il parle tout près, d'un secret. Nino sent un malaise. Son ventre se serre, petit. Je n'aime pas ça. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. Le ventre reste serré. À la sortie, papa attend près des casiers. On rentre, Nino ? Oui. Nino touche l'éclat de casier, un instant. Le soir, la porte de la maison s'ouvre. Une lumière ronde vient de la cuisine. Ça sent le cacao, un peu sucré. L'escalier en bois craque. Nino retire la chaussette trop vite. Elle tombe sur la première marche. Te voilà, Nino. Le cacao est prêt. J'ai quelque chose, maintenant ! Nino avance trop vite vers la cuisine. Maman remue la casserole.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Yasmine est à l'école. La maîtresse parle. Yasmine aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les ciseaux. Yasmine range. Elle écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Yasmine sent un malaise. Son ventre est serré. Le soir, maman l'attend. Yasmine vient raconter à la maison. Elle dit : maman, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute. Maman dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. Le lendemain, Yasmine écoute encore. Un camarade dit : ne le dis pas. Yasmine sent encore un malaise. Le soir, elle raconte à la maison. Même leçon, autre jour. [pause]</t>
+          <t>Les casiers claquent dans le couloir. Le métal est froid, un peu lisse. Sur la porte, un &lt;emphasis&gt;éclat de casier&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le métal ? Nino accroche son manteau. Le crochet fait tic. Une étiquette pend au cartable. Elle est froide sous le doigt. Elle pique un peu. Je reviens te chercher. Oui, papa. Papa serre l'épaule de Nino. Il part vers la porte. Une chaussette bleue dépasse du pantalon. La laine est un peu rêche. Elle chatouille. La classe sent les feuilles. Un banc de bois attend sous la fenêtre. Bonjour. Bonjour, maîtresse. Nino pose le cartable près du banc. Il s'assoit, le dos droit. Un camarade s'approche du banc. Il parle tout près, d'un secret. Nino sent un malaise. Son ventre se serre, petit. Je n'aime pas ça. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le dis, maintenant ! En ce moment, Nino ouvre la bouche. Ses mots se cognent à la classe. Personne ne tourne la tête. Oh. Le sourire de Nino disparaît. Ses épaules tombent un peu. Nino referme la bouche. Les mains restent sur les genoux. Le ventre reste serré. À la sortie, papa attend près des casiers. On rentre, Nino ? Oui. Nino touche l'éclat de casier, un instant. Le soir, la porte de la maison s'ouvre. Une lumière ronde vient de la cuisine. Ça sent le cacao, un peu sucré. L'escalier en bois craque. Nino retire la chaussette trop vite. Elle tombe sur la première marche. Te voilà, Nino. Le cacao est prêt. J'ai quelque chose, maintenant ! Nino avance trop vite vers la cuisine. Maman remue la casserole. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de casier</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,64 +1321,72 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis malaise; intensite=2; destinataire=enfant; sous_texte=il_veut_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une chaussette bleue attend sur la première marche.
-narrateur|L'escalier en bois craque, tout doux.
+          <t>narrateur|Les casiers claquent dans le couloir.
+narrateur|Le métal est froid, un peu lisse.
+narrateur|Sur la porte, un éclat de casier luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le métal ?
+narrateur|Nino accroche son manteau.
+narrateur|Le crochet fait tic.
+narrateur|Une étiquette pend au cartable.
+narrateur|Elle est froide sous le doigt.
+enfant-m|Elle pique un peu.
+papa|Je reviens te chercher.
+enfant-m|Oui, papa.
+narrateur|Papa serre l'épaule de Nino.
+narrateur|Il part vers la porte.
+narrateur|Une chaussette bleue dépasse du pantalon.
+narrateur|La laine est un peu rêche.
+enfant-m|Elle chatouille.
+narrateur|La classe sent les feuilles.
+narrateur|Un banc de bois attend sous la fenêtre.
+maitresse|Bonjour.
+enfant-m|Bonjour, maîtresse.
+narrateur|Nino pose le cartable près du banc.
+narrateur|Il s'assoit, le dos droit.
+narrateur|Un camarade s'approche du banc.
+narrateur|Il parle tout près, d'un secret.
+narrateur|Nino sent un malaise.
+narrateur|Son ventre se serre, petit.
+enfant-m|Je n'aime pas ça.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Je le dis, maintenant !
+narrateur|En ce moment, Nino ouvre la bouche.
+narrateur|Ses mots se cognent à la classe.
+narrateur|Personne ne tourne la tête.
+enfant-m|Oh.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Ses épaules tombent un peu.
+narrateur|Nino referme la bouche.
+narrateur|Les mains restent sur les genoux.
+narrateur|Le ventre reste serré.
+narrateur|À la sortie, papa attend près des casiers.
+papa|On rentre, Nino ?
+enfant-m|Oui.
+narrateur|Nino touche l'éclat de casier, un instant.
+narrateur|Le soir, la porte de la maison s'ouvre.
 narrateur|Une lumière ronde vient de la cuisine.
 narrateur|Ça sent le cacao, un peu sucré.
-narrateur|Maman chante tout bas, près de la casserole.
-narrateur|Papa cherche l'autre chaussette sous le banc.
-papa|La voilà.
-papa|Elle s'était cachée.
-maman|La bleue t'attendait, Nino.
-narrateur|En ce moment, Nino s'assoit pour l'enfiler.
-narrateur|La laine est un peu rêche, un peu chaude.
-enfant-m|Elle chatouille, papa.
-papa|Tire jusqu'au talon.
-papa|Et l'autre.
-narrateur|Nino enfile la deuxième.
-maman|Tes deux pieds sont au chaud.
-enfant-m|Merci, maman.
-enfant-m|À l'école, je veux découper une bande.
-enfant-m|Une bande bleue, comme la chaussette.
-papa|Les ciseaux attendent dans la classe.
-maman|Tu écoutes d'abord.
-enfant-m|Oui.
-narrateur|Nino pose le pied sur la marche.
-narrateur|L'escalier craque encore.
-narrateur|À l'école, la classe sent les feuilles neuves.
-maitresse|Bonjour.
-maitresse|On range les ciseaux.
-enfant-m|Bonjour, maîtresse.
-narrateur|Nino écoute.
-narrateur|Il pose les ciseaux, les pointes en bas.
-maitresse|Maintenant, on découpe une bande.
-narrateur|Nino choisit le papier bleu.
-narrateur|Il découpe tout doux.
-narrateur|La bande tombe, longue et fine.
-enfant-m|Elle ressemble à ma chaussette.
-maitresse|Oui, Nino.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, d'un secret.
-narrateur|Nino sent un malaise.
-narrateur|Son ventre se serre.
-narrateur|Il repose les mains sur ses genoux.
-narrateur|Il reste près de sa chaise.
-narrateur|La bande bleue attend sur la table.
-narrateur|Le soir, la chaussette bleue sèche près du radiateur.
-narrateur|La porte s'ouvre.
-maman|Te voilà.
-maman|Le cacao est prêt.
-narrateur|Nino pose la bande bleue sur la marche.
-narrateur|À côté de l'endroit de ce matin.
-narrateur|Le ventre est encore serré.</t>
+narrateur|L'escalier en bois craque.
+narrateur|Nino retire la chaussette trop vite.
+narrateur|Elle tombe sur la première marche.
+maman|Te voilà, Nino.
+papa|Le cacao est prêt.
+enfant-m|J'ai quelque chose, maintenant !
+narrateur|Nino avance trop vite vers la cuisine.
+narrateur|Maman remue la casserole.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pas,porte</t>
+          <t>casier,pas</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1418,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a un malaise. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Yasmine a un malaise. Que fait-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1425,7 +1433,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | il raconte | à maman | à la maison | écouter</t>
+          <t>raconter | il raconte | à maman | à la maison | près de l'escalier | écouter</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1440,7 +1448,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il raconte à maman. Que fait Nino ?</t>
+          <t>Il raconte près de l'escalier. Que fait Nino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,7 +1486,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,10 +1494,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1512,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,23 +1552,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_raconte_pres_de_l_escalier; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1601,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près du cacao. Nino parle. Maman écoute. Papa écoute. Tu as bien fait. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens raconter. Nino souffle sur le cacao. Une petite fumée danse. Le ventre se desserre, un peu.</t>
+          <t>Nino parle trop vite, près de la porte. Maman, un secret ! Maman n'a pas fini sa phrase. Le cacao fume, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il écoute la cuisine, un instant. Tu veux venir près de l'escalier ? Papa s'accroupit à la même hauteur. Nino pose un pied sur la marche. Le bois est tiède, un peu lisse. La chaussette bleue attend à côté. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as soif ? Un peu, maman. La lumière touche le bois.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Maman. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près du cacao. Nino parle. Maman écoute. Papa écoute. Tu as bien fait. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens raconter. Nino souffle sur le cacao. Une petite fumée danse. Le ventre se desserre, un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino parle trop vite, près de la porte. Maman, un secret ! Maman n'a pas fini sa phrase. Le cacao fume, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il écoute la cuisine, un instant. Tu veux venir près de l'&lt;emphasis level="moderate"&gt;escalier&lt;/emphasis&gt; ? Papa s'accroupit à la même hauteur. Nino pose un pied sur la marche. Le bois est tiède, un peu lisse. La chaussette bleue attend à côté. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as soif ? Un peu, maman. La lumière touche le bois.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Yasmine a écouté la maîtresse. Elle a raconté son malaise à la maison. Maman est là. [pause]</t>
+          <t>Nino parle trop vite, près de la porte. Maman, un secret ! Maman n'a pas fini sa phrase. Le cacao fume, Nino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Il refuse de foncer. Nino referme la bouche. Il écoute la cuisine, un instant. Tu veux venir près de l'&lt;emphasis&gt;escalier&lt;/emphasis&gt; ? Papa s'accroupit à la même hauteur. Nino pose un pied sur la marche. Le bois est tiède, un peu lisse. La chaussette bleue attend à côté. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Tu as soif ? Un peu, maman. La lumière touche le bois. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1658,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1666,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1678,7 +1690,11 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>escalier</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
@@ -1690,16 +1706,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1724,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,25 +1740,41 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_porte_echoue_l_escalier_entend; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Maman.
+          <t>narrateur|Nino parle trop vite, près de la porte.
+enfant-m|Maman, un secret !
+narrateur|Maman n'a pas fini sa phrase.
+maman|Le cacao fume, Nino.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Il refuse de foncer.
+narrateur|Nino referme la bouche.
+narrateur|Il écoute la cuisine, un instant.
+papa|Tu veux venir près de l'escalier ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nino pose un pied sur la marche.
+narrateur|Le bois est tiède, un peu lisse.
+narrateur|La chaussette bleue attend à côté.
 enfant-m|J'ai eu un malaise.
 enfant-m|Quelqu'un a parlé d'un secret.
 maman|On t'écoute.
-papa|Viens près du cacao.
-narrateur|Nino parle.
-narrateur|Maman écoute.
-narrateur|Papa écoute.
-maman|Tu as bien fait.
-papa|À l'école, on écoute la maîtresse.
-maman|Si tu as un malaise, tu viens raconter.
-narrateur|Nino souffle sur le cacao.
-narrateur|Une petite fumée danse.
-narrateur|Le ventre se desserre, un peu.</t>
+papa|Merci, Nino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as soif ?
+enfant-m|Un peu, maman.
+narrateur|La lumière touche le bois.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>cacao,escalier</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1801,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino boit une gorgée. C'est chaud, un peu sucré. Tu as fini ta tasse ? Presque. Maman tient sa main. La main est tiède. Ma bande bleue est sur la marche. On la laisse sécher, comme la chaussette. Le lendemain, l'escalier craque encore. La chaussette bleue attend de nouveau. Même marche. Même chaussette. Tu es prêt ? Je suis prêt, papa. Nino enfile la laine. Elle chatouille encore. Le ventre est calme. On t'écoute, chaque jour. Je le sais.</t>
+          <t>Nino prend la tasse trop vite. Je dis tout, d'un coup ! Le cacao tremble au bord. La chaussette glisse d'un cran. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe la marche, écoute la maison. Sur le cartable, un éclat de casier luit. Là, près de l'escalier. Nino pose d'abord la tasse. Puis il ramasse la laine. Le secret, c'était trop près. Tu veux le dire ici ? Oui, papa. Nino s'assoit sur la marche. Mon ventre s'est serré. On est là. La lumière de la cuisine touche le bois. Nino boit une gorgée. C'est chaud, un peu sucré. Tu as fini ta tasse ? Presque.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino boit une gorgée. C'est chaud, un peu sucré. Tu as fini ta tasse ? Presque. Maman tient sa main. La main est tiède. Ma bande bleue est sur la marche. On la laisse sécher, comme la chaussette. Le lendemain, l'escalier craque encore. La chaussette bleue attend de nouveau. Même marche. Même chaussette. Tu es prêt ? Je suis prêt, papa. Nino enfile la laine. Elle chatouille encore. Le ventre est calme. On t'écoute, chaque jour. Je le sais.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prend la tasse trop vite. Je dis tout, d'un coup ! Le cacao tremble au bord. La chaussette glisse d'un cran. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe la marche, écoute la maison. Sur le cartable, un &lt;emphasis level="moderate"&gt;éclat de casier&lt;/emphasis&gt; luit. Là, près de l'escalier. Nino pose d'abord la tasse. Puis il ramasse la laine. Le secret, c'était trop près. Tu veux le dire ici ? Oui, papa. Nino s'assoit sur la marche. Mon ventre s'est serré. On est là. La lumière de la cuisine touche le bois. Nino boit une gorgée. C'est chaud, un peu sucré. Tu as fini ta tasse ? Presque.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Yasmine boit un verre d'eau. Maman lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Nino prend la tasse trop vite. Je dis tout, d'un coup ! Le cacao tremble au bord. La chaussette glisse d'un cran. Oh. Nino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Nino observe la marche, écoute la maison. Sur le cartable, un &lt;emphasis&gt;éclat de casier&lt;/emphasis&gt; luit. Là, près de l'escalier. Nino pose d'abord la tasse. Puis il ramasse la laine. Le secret, c'était trop près. Tu veux le dire ici ? Oui, papa. Nino s'assoit sur la marche. Mon ventre s'est serré. On est là. La lumière de la cuisine touche le bois. Nino boit une gorgée. C'est chaud, un peu sucré. Tu as fini ta tasse ? Presque. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1826,7 +1858,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1834,10 +1866,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1860,30 +1892,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de casier</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1892,10 +1924,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1906,28 +1938,43 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino boit une gorgée.
+          <t>narrateur|Nino prend la tasse trop vite.
+enfant-m|Je dis tout, d'un coup !
+narrateur|Le cacao tremble au bord.
+narrateur|La chaussette glisse d'un cran.
+enfant-m|Oh.
+narrateur|Nino avance les mains.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Nino observe la marche, écoute la maison.
+narrateur|Sur le cartable, un éclat de casier luit.
+enfant-m|Là, près de l'escalier.
+narrateur|Nino pose d'abord la tasse.
+narrateur|Puis il ramasse la laine.
+enfant-m|Le secret, c'était trop près.
+papa|Tu veux le dire ici ?
+enfant-m|Oui, papa.
+narrateur|Nino s'assoit sur la marche.
+enfant-m|Mon ventre s'est serré.
+maman|On est là.
+narrateur|La lumière de la cuisine touche le bois.
+narrateur|Nino boit une gorgée.
 narrateur|C'est chaud, un peu sucré.
 papa|Tu as fini ta tasse ?
-enfant-m|Presque.
-narrateur|Maman tient sa main.
-narrateur|La main est tiède.
-enfant-m|Ma bande bleue est sur la marche.
-maman|On la laisse sécher, comme la chaussette.
-narrateur|Le lendemain, l'escalier craque encore.
-narrateur|La chaussette bleue attend de nouveau.
-papa|Même marche.
-papa|Même chaussette.
-papa|Tu es prêt ?
-enfant-m|Je suis prêt, papa.
-narrateur|Nino enfile la laine.
-narrateur|Elle chatouille encore.
-narrateur|Le ventre est calme.
-maman|On t'écoute, chaque jour.
-enfant-m|Je le sais.</t>
+enfant-m|Presque.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>tasse,laine</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2001,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La bande bleue reste près du radiateur. La chaussette aussi. On t'a écouté, Nino. Le cacao a attendu.</t>
+          <t>Le casier brillait, papa. Tu le vois, comme ce matin ? Oui, sur le métal. Nino pose la chaussette sur la marche. On la laisse là ? Oui, maman. La lumière de la cuisine touche la laine. Une vapeur monte du cacao. Nino respire, plus large. L'escalier en bois se tait. Un éclat de casier reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La bande bleue reste près du radiateur. La chaussette aussi. On t'a écouté, Nino. Le cacao a attendu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le casier brillait, papa. Tu le vois, comme ce matin ? Oui, sur le métal. Nino pose la chaussette sur la marche. On la laisse là ? Oui, maman. La lumière de la cuisine touche la laine. Une vapeur monte du cacao. Nino respire, plus large. L'escalier en bois se tait. Un &lt;emphasis level="moderate"&gt;éclat de casier&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le casier brillait, papa. Tu le vois, comme ce matin ? Oui, sur le métal. Nino pose la chaussette sur la marche. On la laisse là ? Oui, maman. La lumière de la cuisine touche la laine. Une vapeur monte du cacao. Nino respire, plus large. L'escalier en bois se tait. Un &lt;emphasis&gt;éclat de casier&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,7 +2058,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2019,10 +2066,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2078,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2092,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de casier</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2115,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,27 +2128,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La bande bleue reste près du radiateur.
-narrateur|La chaussette aussi.
-papa|On t'a écouté, Nino.
-maman|Le cacao a attendu.</t>
+          <t>enfant-m|Le casier brillait, papa.
+papa|Tu le vois, comme ce matin ?
+enfant-m|Oui, sur le métal.
+narrateur|Nino pose la chaussette sur la marche.
+maman|On la laisse là ?
+enfant-m|Oui, maman.
+narrateur|La lumière de la cuisine touche la laine.
+narrateur|Une vapeur monte du cacao.
+narrateur|Nino respire, plus large.
+narrateur|L'escalier en bois se tait.
+narrateur|Un éclat de casier reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>casier,cacao</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2175,6 +2242,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>